<commit_message>
Day 3 of Learning Excel
</commit_message>
<xml_diff>
--- a/Day 3 Excel.xlsx
+++ b/Day 3 Excel.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Naik Balkrushna Anil\OneDrive\Attachments\Desktop\Exploring Data Science Field\Basic of Excel\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Naik Balkrushna Anil\OneDrive\Attachments\Desktop\Full Stack Development\Exploring Data Science Field\Basic of Excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7D4E0AEA-25E8-426B-94E2-CB56DD65E1E1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7DAB3016-2082-4A1A-8EC4-7264A99E989A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="21">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="63" uniqueCount="29">
   <si>
     <t xml:space="preserve">Name </t>
   </si>
@@ -45,9 +45,6 @@
     <t>English</t>
   </si>
   <si>
-    <t>Total Marks</t>
-  </si>
-  <si>
     <t>Day 3: Absolute References in Excel</t>
   </si>
   <si>
@@ -88,13 +85,40 @@
   </si>
   <si>
     <t>Evaluate Formula</t>
+  </si>
+  <si>
+    <t>Day 3: Functions in Excel</t>
+  </si>
+  <si>
+    <t>Total Marks of Harshali</t>
+  </si>
+  <si>
+    <t>Total Marks of Madhu</t>
+  </si>
+  <si>
+    <t>Average of Marathi</t>
+  </si>
+  <si>
+    <t>Average of English</t>
+  </si>
+  <si>
+    <t>Percentage of Jaya</t>
+  </si>
+  <si>
+    <t>Day 3: Commonly Used Excel Functions</t>
+  </si>
+  <si>
+    <t>Min</t>
+  </si>
+  <si>
+    <t>Max</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -117,6 +141,12 @@
       <color theme="1"/>
       <name val="Roboto"/>
     </font>
+    <font>
+      <b/>
+      <sz val="16"/>
+      <color theme="1"/>
+      <name val="Roboto"/>
+    </font>
   </fonts>
   <fills count="3">
     <fill>
@@ -132,7 +162,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="7">
+  <borders count="13">
     <border>
       <left/>
       <right/>
@@ -216,11 +246,73 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="28">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -234,26 +326,63 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -536,34 +665,34 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:P14"/>
+  <dimension ref="A1:R38"/>
   <sheetFormatPr defaultColWidth="10.33203125" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="10.33203125" customWidth="1"/>
+    <col min="8" max="8" width="21.21875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A1" s="12" t="s">
-        <v>7</v>
-      </c>
-      <c r="B1" s="12"/>
-      <c r="C1" s="12"/>
-      <c r="D1" s="12"/>
-      <c r="E1" s="12"/>
-      <c r="F1" s="12"/>
-      <c r="G1" s="12"/>
-      <c r="H1" s="12" t="s">
-        <v>19</v>
-      </c>
-      <c r="I1" s="12"/>
-      <c r="J1" s="12"/>
-      <c r="K1" s="12"/>
-      <c r="L1" s="12"/>
-      <c r="M1" s="12"/>
-      <c r="N1" s="12"/>
-    </row>
-    <row r="2" spans="1:16" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
-    <row r="3" spans="1:16" ht="28.2" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:15" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A1" s="9" t="s">
+        <v>6</v>
+      </c>
+      <c r="B1" s="9"/>
+      <c r="C1" s="9"/>
+      <c r="D1" s="9"/>
+      <c r="E1" s="9"/>
+      <c r="F1" s="9"/>
+      <c r="G1" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="H1" s="9"/>
+      <c r="I1" s="9"/>
+      <c r="J1" s="9"/>
+      <c r="K1" s="9"/>
+      <c r="L1" s="9"/>
+      <c r="M1" s="9"/>
+    </row>
+    <row r="2" spans="1:15" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
+    <row r="3" spans="1:15" ht="28.2" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A3" s="3" t="s">
         <v>0</v>
       </c>
@@ -582,63 +711,56 @@
       <c r="F3" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="G3" s="5" t="s">
-        <v>6</v>
+      <c r="H3">
+        <v>56</v>
       </c>
       <c r="I3">
-        <v>56</v>
+        <v>34</v>
       </c>
       <c r="J3">
-        <v>34</v>
+        <v>67</v>
       </c>
       <c r="K3">
-        <v>67</v>
+        <v>87</v>
       </c>
       <c r="L3">
-        <v>87</v>
+        <v>65</v>
       </c>
       <c r="M3">
-        <v>65</v>
+        <f>1+5*J3</f>
+        <v>336</v>
       </c>
       <c r="N3">
-        <f>1+5*K3</f>
-        <v>336</v>
-      </c>
-      <c r="O3">
-        <f>3*45/10*56-K3+67</f>
+        <f>3*45/10*56-J3+67</f>
         <v>756</v>
       </c>
-      <c r="P3" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="4" spans="1:16" ht="27.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="O3" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="4" spans="1:15" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="B4" s="5">
+        <v>86</v>
+      </c>
+      <c r="C4" s="5">
+        <v>89</v>
+      </c>
+      <c r="D4" s="5">
+        <v>98</v>
+      </c>
+      <c r="E4" s="5">
+        <v>86</v>
+      </c>
+      <c r="F4" s="5">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="5" spans="1:15" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="1" t="s">
         <v>8</v>
-      </c>
-      <c r="B4" s="6">
-        <v>86</v>
-      </c>
-      <c r="C4" s="6">
-        <v>89</v>
-      </c>
-      <c r="D4" s="6">
-        <v>98</v>
-      </c>
-      <c r="E4" s="6">
-        <v>86</v>
-      </c>
-      <c r="F4" s="6">
-        <v>89</v>
-      </c>
-      <c r="G4" s="6">
-        <f>B4+C4+D4+E4+F4</f>
-        <v>448</v>
-      </c>
-    </row>
-    <row r="5" spans="1:16" ht="27.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A5" s="1" t="s">
-        <v>9</v>
       </c>
       <c r="B5" s="1">
         <v>89</v>
@@ -655,14 +777,10 @@
       <c r="F5" s="1">
         <v>87</v>
       </c>
-      <c r="G5" s="6">
-        <f t="shared" ref="G5:G13" si="0">B5+C5+D5+E5+F5</f>
-        <v>430</v>
-      </c>
-    </row>
-    <row r="6" spans="1:16" ht="27.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    </row>
+    <row r="6" spans="1:15" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="1" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B6" s="1">
         <v>78</v>
@@ -679,158 +797,130 @@
       <c r="F6" s="1">
         <v>67</v>
       </c>
-      <c r="G6" s="6">
-        <f t="shared" si="0"/>
-        <v>386</v>
-      </c>
-    </row>
-    <row r="7" spans="1:16" ht="27.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    </row>
+    <row r="7" spans="1:15" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="B7" s="1">
+        <v>68</v>
+      </c>
+      <c r="C7" s="1">
+        <v>65</v>
+      </c>
+      <c r="D7" s="1">
+        <v>93</v>
+      </c>
+      <c r="E7" s="1">
+        <v>68</v>
+      </c>
+      <c r="F7" s="1">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="8" spans="1:15" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="B7" s="7">
-        <v>68</v>
-      </c>
-      <c r="C7" s="7">
-        <v>65</v>
-      </c>
-      <c r="D7" s="7">
-        <v>93</v>
-      </c>
-      <c r="E7" s="7">
-        <v>68</v>
-      </c>
-      <c r="F7" s="7">
-        <v>65</v>
-      </c>
-      <c r="G7" s="6">
-        <f t="shared" si="0"/>
-        <v>359</v>
-      </c>
-    </row>
-    <row r="8" spans="1:16" ht="27.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A8" s="1" t="s">
+      <c r="B8" s="1">
+        <v>94</v>
+      </c>
+      <c r="C8" s="1">
+        <v>47</v>
+      </c>
+      <c r="D8" s="1">
+        <v>89</v>
+      </c>
+      <c r="E8" s="1">
+        <v>94</v>
+      </c>
+      <c r="F8" s="1">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="9" spans="1:15" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A9" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="B8" s="7">
-        <v>94</v>
-      </c>
-      <c r="C8" s="7">
+      <c r="B9" s="1">
+        <v>89</v>
+      </c>
+      <c r="C9" s="1">
+        <v>78</v>
+      </c>
+      <c r="D9" s="1">
+        <v>81</v>
+      </c>
+      <c r="E9" s="1">
+        <v>89</v>
+      </c>
+      <c r="F9" s="1">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="10" spans="1:15" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A10" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="B10" s="1">
+        <v>74</v>
+      </c>
+      <c r="C10" s="1">
+        <v>98</v>
+      </c>
+      <c r="D10" s="1">
+        <v>72</v>
+      </c>
+      <c r="E10" s="1">
+        <v>74</v>
+      </c>
+      <c r="F10" s="1">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="11" spans="1:15" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A11" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="B11" s="1">
+        <v>84</v>
+      </c>
+      <c r="C11" s="1">
+        <v>78</v>
+      </c>
+      <c r="D11" s="1">
+        <v>84</v>
+      </c>
+      <c r="E11" s="1">
+        <v>84</v>
+      </c>
+      <c r="F11" s="1">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="12" spans="1:15" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A12" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="B12" s="1">
         <v>47</v>
       </c>
-      <c r="D8" s="7">
-        <v>89</v>
-      </c>
-      <c r="E8" s="7">
-        <v>94</v>
-      </c>
-      <c r="F8" s="7">
+      <c r="C12" s="1">
+        <v>67</v>
+      </c>
+      <c r="D12" s="1">
+        <v>98</v>
+      </c>
+      <c r="E12" s="1">
         <v>47</v>
       </c>
-      <c r="G8" s="6">
-        <f t="shared" si="0"/>
-        <v>371</v>
-      </c>
-    </row>
-    <row r="9" spans="1:16" ht="27.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A9" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="B9" s="7">
-        <v>89</v>
-      </c>
-      <c r="C9" s="7">
-        <v>78</v>
-      </c>
-      <c r="D9" s="7">
-        <v>81</v>
-      </c>
-      <c r="E9" s="7">
-        <v>89</v>
-      </c>
-      <c r="F9" s="7">
-        <v>78</v>
-      </c>
-      <c r="G9" s="6">
-        <f t="shared" si="0"/>
-        <v>415</v>
-      </c>
-    </row>
-    <row r="10" spans="1:16" ht="27.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A10" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="B10" s="7">
-        <v>74</v>
-      </c>
-      <c r="C10" s="7">
-        <v>98</v>
-      </c>
-      <c r="D10" s="7">
-        <v>72</v>
-      </c>
-      <c r="E10" s="7">
-        <v>74</v>
-      </c>
-      <c r="F10" s="7">
-        <v>98</v>
-      </c>
-      <c r="G10" s="6">
-        <f t="shared" si="0"/>
-        <v>416</v>
-      </c>
-    </row>
-    <row r="11" spans="1:16" ht="27.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A11" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="B11" s="7">
-        <v>84</v>
-      </c>
-      <c r="C11" s="7">
-        <v>78</v>
-      </c>
-      <c r="D11" s="7">
-        <v>84</v>
-      </c>
-      <c r="E11" s="7">
-        <v>84</v>
-      </c>
-      <c r="F11" s="7">
-        <v>78</v>
-      </c>
-      <c r="G11" s="6">
-        <f t="shared" si="0"/>
-        <v>408</v>
-      </c>
-    </row>
-    <row r="12" spans="1:16" ht="27.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A12" s="1" t="s">
+      <c r="F12" s="1">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="13" spans="1:15" ht="27.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A13" s="2" t="s">
         <v>16</v>
-      </c>
-      <c r="B12" s="7">
-        <v>47</v>
-      </c>
-      <c r="C12" s="7">
-        <v>67</v>
-      </c>
-      <c r="D12" s="7">
-        <v>98</v>
-      </c>
-      <c r="E12" s="7">
-        <v>47</v>
-      </c>
-      <c r="F12" s="7">
-        <v>67</v>
-      </c>
-      <c r="G12" s="6">
-        <f t="shared" si="0"/>
-        <v>326</v>
-      </c>
-    </row>
-    <row r="13" spans="1:16" ht="27.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A13" s="2" t="s">
-        <v>17</v>
       </c>
       <c r="B13" s="2">
         <v>90</v>
@@ -847,44 +937,628 @@
       <c r="F13" s="2">
         <v>59</v>
       </c>
-      <c r="G13" s="8">
+    </row>
+    <row r="14" spans="1:15" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A14" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="B14" s="8">
+        <f t="shared" ref="B14:F14" si="0">AVERAGE(B4:B13)</f>
+        <v>79.900000000000006</v>
+      </c>
+      <c r="C14" s="8">
         <f t="shared" si="0"/>
-        <v>387</v>
-      </c>
-    </row>
-    <row r="14" spans="1:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A14" s="10" t="s">
-        <v>18</v>
-      </c>
-      <c r="B14" s="11">
-        <f>AVERAGE(B4:B13)</f>
+        <v>73.5</v>
+      </c>
+      <c r="D14" s="8">
+        <f t="shared" si="0"/>
+        <v>87.8</v>
+      </c>
+      <c r="E14" s="8">
+        <f t="shared" si="0"/>
         <v>79.900000000000006</v>
       </c>
-      <c r="C14" s="11">
-        <f>AVERAGE(C4:C13)</f>
+      <c r="F14" s="8">
+        <f t="shared" si="0"/>
         <v>73.5</v>
       </c>
-      <c r="D14" s="11">
-        <f>AVERAGE(D4:D13)</f>
+    </row>
+    <row r="17" spans="1:18" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A17" s="10" t="s">
+        <v>20</v>
+      </c>
+      <c r="B17" s="11"/>
+      <c r="C17" s="11"/>
+      <c r="D17" s="11"/>
+      <c r="E17" s="11"/>
+      <c r="F17" s="11"/>
+      <c r="M17" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="N17" s="10"/>
+      <c r="O17" s="10"/>
+      <c r="P17" s="10"/>
+      <c r="Q17" s="10"/>
+      <c r="R17" s="10"/>
+    </row>
+    <row r="18" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A18" s="11"/>
+      <c r="B18" s="11"/>
+      <c r="C18" s="11"/>
+      <c r="D18" s="11"/>
+      <c r="E18" s="11"/>
+      <c r="F18" s="11"/>
+      <c r="M18" s="10"/>
+      <c r="N18" s="10"/>
+      <c r="O18" s="10"/>
+      <c r="P18" s="10"/>
+      <c r="Q18" s="10"/>
+      <c r="R18" s="10"/>
+    </row>
+    <row r="19" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A19" t="s">
+        <v>0</v>
+      </c>
+      <c r="B19" t="s">
+        <v>1</v>
+      </c>
+      <c r="C19" t="s">
+        <v>2</v>
+      </c>
+      <c r="D19" t="s">
+        <v>3</v>
+      </c>
+      <c r="E19" t="s">
+        <v>4</v>
+      </c>
+      <c r="F19" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="20" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A20" t="s">
+        <v>7</v>
+      </c>
+      <c r="B20">
+        <v>86</v>
+      </c>
+      <c r="C20">
+        <v>89</v>
+      </c>
+      <c r="D20">
+        <v>98</v>
+      </c>
+      <c r="E20">
+        <v>86</v>
+      </c>
+      <c r="F20">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="21" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A21" t="s">
+        <v>8</v>
+      </c>
+      <c r="B21">
+        <v>89</v>
+      </c>
+      <c r="C21">
+        <v>87</v>
+      </c>
+      <c r="D21">
+        <v>78</v>
+      </c>
+      <c r="E21">
+        <v>89</v>
+      </c>
+      <c r="F21">
+        <v>87</v>
+      </c>
+      <c r="M21" s="6" t="s">
+        <v>0</v>
+      </c>
+      <c r="N21" s="16" t="s">
+        <v>1</v>
+      </c>
+      <c r="O21" s="16" t="s">
+        <v>2</v>
+      </c>
+      <c r="P21" s="16" t="s">
+        <v>3</v>
+      </c>
+      <c r="Q21" s="16" t="s">
+        <v>4</v>
+      </c>
+      <c r="R21" s="17" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="22" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A22" t="s">
+        <v>9</v>
+      </c>
+      <c r="B22">
+        <v>78</v>
+      </c>
+      <c r="C22">
+        <v>67</v>
+      </c>
+      <c r="D22">
+        <v>96</v>
+      </c>
+      <c r="E22">
+        <v>78</v>
+      </c>
+      <c r="F22">
+        <v>67</v>
+      </c>
+      <c r="M22" s="18" t="s">
+        <v>7</v>
+      </c>
+      <c r="N22" s="19">
+        <v>86</v>
+      </c>
+      <c r="O22" s="19">
+        <v>89</v>
+      </c>
+      <c r="P22" s="19">
+        <v>98</v>
+      </c>
+      <c r="Q22" s="19">
+        <v>86</v>
+      </c>
+      <c r="R22" s="20">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="23" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A23" t="s">
+        <v>10</v>
+      </c>
+      <c r="B23">
+        <v>68</v>
+      </c>
+      <c r="C23">
+        <v>65</v>
+      </c>
+      <c r="D23">
+        <v>93</v>
+      </c>
+      <c r="E23">
+        <v>68</v>
+      </c>
+      <c r="F23">
+        <v>65</v>
+      </c>
+      <c r="M23" s="18" t="s">
+        <v>8</v>
+      </c>
+      <c r="N23" s="19">
+        <v>89</v>
+      </c>
+      <c r="O23" s="19">
+        <v>87</v>
+      </c>
+      <c r="P23" s="19">
+        <v>78</v>
+      </c>
+      <c r="Q23" s="19">
+        <v>89</v>
+      </c>
+      <c r="R23" s="20">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="24" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A24" t="s">
+        <v>11</v>
+      </c>
+      <c r="B24">
+        <v>94</v>
+      </c>
+      <c r="C24">
+        <v>47</v>
+      </c>
+      <c r="D24">
+        <v>89</v>
+      </c>
+      <c r="E24">
+        <v>94</v>
+      </c>
+      <c r="F24">
+        <v>47</v>
+      </c>
+      <c r="M24" s="18" t="s">
+        <v>9</v>
+      </c>
+      <c r="N24" s="19">
+        <v>78</v>
+      </c>
+      <c r="O24" s="19">
+        <v>67</v>
+      </c>
+      <c r="P24" s="19">
+        <v>96</v>
+      </c>
+      <c r="Q24" s="19">
+        <v>78</v>
+      </c>
+      <c r="R24" s="20">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="25" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A25" t="s">
+        <v>12</v>
+      </c>
+      <c r="B25">
+        <v>89</v>
+      </c>
+      <c r="C25">
+        <v>78</v>
+      </c>
+      <c r="D25">
+        <v>81</v>
+      </c>
+      <c r="E25">
+        <v>89</v>
+      </c>
+      <c r="F25">
+        <v>78</v>
+      </c>
+      <c r="M25" s="18" t="s">
+        <v>10</v>
+      </c>
+      <c r="N25" s="19">
+        <v>68</v>
+      </c>
+      <c r="O25" s="19">
+        <v>65</v>
+      </c>
+      <c r="P25" s="19">
+        <v>93</v>
+      </c>
+      <c r="Q25" s="19">
+        <v>68</v>
+      </c>
+      <c r="R25" s="20">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="26" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A26" t="s">
+        <v>13</v>
+      </c>
+      <c r="B26">
+        <v>74</v>
+      </c>
+      <c r="C26">
+        <v>98</v>
+      </c>
+      <c r="D26">
+        <v>72</v>
+      </c>
+      <c r="E26">
+        <v>74</v>
+      </c>
+      <c r="F26">
+        <v>98</v>
+      </c>
+      <c r="M26" s="18" t="s">
+        <v>11</v>
+      </c>
+      <c r="N26" s="19">
+        <v>94</v>
+      </c>
+      <c r="O26" s="19">
+        <v>47</v>
+      </c>
+      <c r="P26" s="19">
+        <v>89</v>
+      </c>
+      <c r="Q26" s="19">
+        <v>94</v>
+      </c>
+      <c r="R26" s="20">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="27" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A27" t="s">
+        <v>14</v>
+      </c>
+      <c r="B27">
+        <v>84</v>
+      </c>
+      <c r="C27">
+        <v>78</v>
+      </c>
+      <c r="D27">
+        <v>84</v>
+      </c>
+      <c r="E27">
+        <v>84</v>
+      </c>
+      <c r="F27">
+        <v>78</v>
+      </c>
+      <c r="M27" s="18" t="s">
+        <v>12</v>
+      </c>
+      <c r="N27" s="19">
+        <v>89</v>
+      </c>
+      <c r="O27" s="19">
+        <v>78</v>
+      </c>
+      <c r="P27" s="19">
+        <v>81</v>
+      </c>
+      <c r="Q27" s="19">
+        <v>89</v>
+      </c>
+      <c r="R27" s="20">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="28" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A28" t="s">
+        <v>15</v>
+      </c>
+      <c r="B28">
+        <v>47</v>
+      </c>
+      <c r="C28">
+        <v>67</v>
+      </c>
+      <c r="D28">
+        <v>98</v>
+      </c>
+      <c r="E28">
+        <v>47</v>
+      </c>
+      <c r="F28">
+        <v>67</v>
+      </c>
+      <c r="M28" s="18" t="s">
+        <v>13</v>
+      </c>
+      <c r="N28" s="19">
+        <v>74</v>
+      </c>
+      <c r="O28" s="19">
+        <v>98</v>
+      </c>
+      <c r="P28" s="19">
+        <v>72</v>
+      </c>
+      <c r="Q28" s="19">
+        <v>74</v>
+      </c>
+      <c r="R28" s="20">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="29" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A29" t="s">
+        <v>16</v>
+      </c>
+      <c r="B29">
+        <v>90</v>
+      </c>
+      <c r="C29">
+        <v>59</v>
+      </c>
+      <c r="D29">
+        <v>89</v>
+      </c>
+      <c r="E29">
+        <v>90</v>
+      </c>
+      <c r="F29">
+        <v>59</v>
+      </c>
+      <c r="M29" s="18" t="s">
+        <v>14</v>
+      </c>
+      <c r="N29" s="19">
+        <v>84</v>
+      </c>
+      <c r="O29" s="19">
+        <v>78</v>
+      </c>
+      <c r="P29" s="19">
+        <v>84</v>
+      </c>
+      <c r="Q29" s="19">
+        <v>84</v>
+      </c>
+      <c r="R29" s="20">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="30" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A30" t="s">
+        <v>17</v>
+      </c>
+      <c r="B30">
+        <f t="shared" ref="B30" si="1">AVERAGE(B20:B29)</f>
+        <v>79.900000000000006</v>
+      </c>
+      <c r="C30">
+        <f t="shared" ref="C30" si="2">AVERAGE(C20:C29)</f>
+        <v>73.5</v>
+      </c>
+      <c r="D30">
+        <f t="shared" ref="D30" si="3">AVERAGE(D20:D29)</f>
         <v>87.8</v>
       </c>
-      <c r="E14" s="11">
-        <f>AVERAGE(E4:E13)</f>
+      <c r="E30">
+        <f t="shared" ref="E30" si="4">AVERAGE(E20:E29)</f>
         <v>79.900000000000006</v>
       </c>
-      <c r="F14" s="11">
-        <f>AVERAGE(F4:F13)</f>
+      <c r="F30">
+        <f t="shared" ref="F30" si="5">AVERAGE(F20:F29)</f>
         <v>73.5</v>
       </c>
-      <c r="G14" s="9">
-        <f>AVERAGE(G4:G13)</f>
-        <v>394.6</v>
+      <c r="M30" s="18" t="s">
+        <v>15</v>
+      </c>
+      <c r="N30" s="19">
+        <v>47</v>
+      </c>
+      <c r="O30" s="19">
+        <v>67</v>
+      </c>
+      <c r="P30" s="19">
+        <v>98</v>
+      </c>
+      <c r="Q30" s="19">
+        <v>47</v>
+      </c>
+      <c r="R30" s="20">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="31" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="M31" s="18" t="s">
+        <v>16</v>
+      </c>
+      <c r="N31" s="19">
+        <v>90</v>
+      </c>
+      <c r="O31" s="19">
+        <v>59</v>
+      </c>
+      <c r="P31" s="19">
+        <v>89</v>
+      </c>
+      <c r="Q31" s="19">
+        <v>90</v>
+      </c>
+      <c r="R31" s="20">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="32" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="H32" s="12" t="s">
+        <v>21</v>
+      </c>
+      <c r="I32" s="13">
+        <f>SUM(20:20)</f>
+        <v>448</v>
+      </c>
+      <c r="M32" s="21" t="s">
+        <v>17</v>
+      </c>
+      <c r="N32" s="22">
+        <f t="shared" ref="N32" si="6">AVERAGE(N22:N31)</f>
+        <v>79.900000000000006</v>
+      </c>
+      <c r="O32" s="22">
+        <f t="shared" ref="O32" si="7">AVERAGE(O22:O31)</f>
+        <v>73.5</v>
+      </c>
+      <c r="P32" s="22">
+        <f t="shared" ref="P32" si="8">AVERAGE(P22:P31)</f>
+        <v>87.8</v>
+      </c>
+      <c r="Q32" s="22">
+        <f t="shared" ref="Q32" si="9">AVERAGE(Q22:Q31)</f>
+        <v>79.900000000000006</v>
+      </c>
+      <c r="R32" s="23">
+        <f t="shared" ref="R32" si="10">AVERAGE(R22:R31)</f>
+        <v>73.5</v>
+      </c>
+    </row>
+    <row r="33" spans="8:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="H33" s="14" t="s">
+        <v>22</v>
+      </c>
+      <c r="I33" s="15"/>
+      <c r="M33" s="24" t="s">
+        <v>27</v>
+      </c>
+      <c r="N33" s="22">
+        <f>MIN(N22:N31)</f>
+        <v>47</v>
+      </c>
+      <c r="O33" s="22">
+        <f t="shared" ref="O33:R33" si="11">MIN(O22:O31)</f>
+        <v>47</v>
+      </c>
+      <c r="P33" s="22">
+        <f t="shared" si="11"/>
+        <v>72</v>
+      </c>
+      <c r="Q33" s="22">
+        <f t="shared" si="11"/>
+        <v>47</v>
+      </c>
+      <c r="R33" s="23">
+        <f t="shared" si="11"/>
+        <v>47</v>
+      </c>
+    </row>
+    <row r="34" spans="8:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="M34" s="25" t="s">
+        <v>28</v>
+      </c>
+      <c r="N34" s="26">
+        <f>MAX(N22:N31)</f>
+        <v>94</v>
+      </c>
+      <c r="O34" s="26">
+        <f t="shared" ref="O34:R34" si="12">MAX(O22:O31)</f>
+        <v>98</v>
+      </c>
+      <c r="P34" s="26">
+        <f t="shared" si="12"/>
+        <v>98</v>
+      </c>
+      <c r="Q34" s="26">
+        <f t="shared" si="12"/>
+        <v>94</v>
+      </c>
+      <c r="R34" s="27">
+        <f t="shared" si="12"/>
+        <v>98</v>
+      </c>
+    </row>
+    <row r="35" spans="8:18" x14ac:dyDescent="0.3">
+      <c r="H35" s="12" t="s">
+        <v>23</v>
+      </c>
+      <c r="I35" s="13">
+        <f>AVERAGE(B20:B30)</f>
+        <v>79.899999999999991</v>
+      </c>
+    </row>
+    <row r="36" spans="8:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="H36" s="14" t="s">
+        <v>24</v>
+      </c>
+      <c r="I36" s="15">
+        <f>AVERAGE(F20:F30)</f>
+        <v>73.5</v>
+      </c>
+    </row>
+    <row r="38" spans="8:18" x14ac:dyDescent="0.3">
+      <c r="H38" t="s">
+        <v>25</v>
+      </c>
+      <c r="I38" t="e">
+        <f>PERCENTILE(B22:F22,100)</f>
+        <v>#NUM!</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="2">
-    <mergeCell ref="A1:G1"/>
-    <mergeCell ref="H1:N1"/>
+  <mergeCells count="4">
+    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="G1:M1"/>
+    <mergeCell ref="A17:F18"/>
+    <mergeCell ref="M17:R18"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>